<commit_message>
Update ⚙️ Configurações do Sistema “calculadora_simples”
</commit_message>
<xml_diff>
--- a/img/calculadora-simples-nacional-configuracoes.xlsx
+++ b/img/calculadora-simples-nacional-configuracoes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thais Camilo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D3A8BFE-5BF1-4569-80E1-DB6E8E6670B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC1FD151-7AEC-43ED-B4BF-07A700DDD644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculadora Simples Nacional" sheetId="1" r:id="rId1"/>
@@ -882,7 +882,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>3600000</v>
+        <v>3700000</v>
       </c>
       <c r="D6">
         <v>0.14299999999999999</v>
@@ -899,7 +899,7 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>4800000</v>
+        <v>5800000</v>
       </c>
       <c r="D7">
         <v>0.19</v>
@@ -916,6 +916,7 @@
         <v>1</v>
       </c>
       <c r="C8">
+        <f>C$2</f>
         <v>180000</v>
       </c>
       <c r="D8">
@@ -933,6 +934,7 @@
         <v>2</v>
       </c>
       <c r="C9">
+        <f>C$3</f>
         <v>360000</v>
       </c>
       <c r="D9">
@@ -950,6 +952,7 @@
         <v>3</v>
       </c>
       <c r="C10">
+        <f>C$4</f>
         <v>720000</v>
       </c>
       <c r="D10">
@@ -967,6 +970,7 @@
         <v>4</v>
       </c>
       <c r="C11">
+        <f>C$5</f>
         <v>1800000</v>
       </c>
       <c r="D11">
@@ -984,7 +988,8 @@
         <v>5</v>
       </c>
       <c r="C12">
-        <v>3600000</v>
+        <f>C$6</f>
+        <v>3700000</v>
       </c>
       <c r="D12">
         <v>0.14699999999999999</v>
@@ -1001,7 +1006,8 @@
         <v>6</v>
       </c>
       <c r="C13">
-        <v>4800000</v>
+        <f>C$7</f>
+        <v>5800000</v>
       </c>
       <c r="D13">
         <v>0.3</v>
@@ -1018,6 +1024,7 @@
         <v>1</v>
       </c>
       <c r="C14">
+        <f>C$2</f>
         <v>180000</v>
       </c>
       <c r="D14">
@@ -1035,6 +1042,7 @@
         <v>2</v>
       </c>
       <c r="C15">
+        <f>C$3</f>
         <v>360000</v>
       </c>
       <c r="D15">
@@ -1052,6 +1060,7 @@
         <v>3</v>
       </c>
       <c r="C16">
+        <f>C$4</f>
         <v>720000</v>
       </c>
       <c r="D16">
@@ -1069,6 +1078,7 @@
         <v>4</v>
       </c>
       <c r="C17">
+        <f>C$5</f>
         <v>1800000</v>
       </c>
       <c r="D17">
@@ -1086,7 +1096,8 @@
         <v>5</v>
       </c>
       <c r="C18">
-        <v>3600000</v>
+        <f>C$6</f>
+        <v>3700000</v>
       </c>
       <c r="D18">
         <v>0.21</v>
@@ -1103,7 +1114,8 @@
         <v>6</v>
       </c>
       <c r="C19">
-        <v>4800000</v>
+        <f>C$7</f>
+        <v>5800000</v>
       </c>
       <c r="D19">
         <v>0.33</v>
@@ -1120,6 +1132,7 @@
         <v>1</v>
       </c>
       <c r="C20">
+        <f>C$2</f>
         <v>180000</v>
       </c>
       <c r="D20">
@@ -1137,6 +1150,7 @@
         <v>2</v>
       </c>
       <c r="C21">
+        <f>C$3</f>
         <v>360000</v>
       </c>
       <c r="D21">
@@ -1154,6 +1168,7 @@
         <v>3</v>
       </c>
       <c r="C22">
+        <f>C$4</f>
         <v>720000</v>
       </c>
       <c r="D22">
@@ -1171,6 +1186,7 @@
         <v>4</v>
       </c>
       <c r="C23">
+        <f>C$5</f>
         <v>1800000</v>
       </c>
       <c r="D23">
@@ -1188,7 +1204,8 @@
         <v>5</v>
       </c>
       <c r="C24">
-        <v>3600000</v>
+        <f>C$6</f>
+        <v>3700000</v>
       </c>
       <c r="D24">
         <v>0.22</v>
@@ -1205,7 +1222,8 @@
         <v>6</v>
       </c>
       <c r="C25">
-        <v>4800000</v>
+        <f>C$7</f>
+        <v>5800000</v>
       </c>
       <c r="D25">
         <v>0.33</v>
@@ -1222,6 +1240,7 @@
         <v>1</v>
       </c>
       <c r="C26">
+        <f>C$2</f>
         <v>180000</v>
       </c>
       <c r="D26">
@@ -1239,6 +1258,7 @@
         <v>2</v>
       </c>
       <c r="C27">
+        <f>C$3</f>
         <v>360000</v>
       </c>
       <c r="D27">
@@ -1256,6 +1276,7 @@
         <v>3</v>
       </c>
       <c r="C28">
+        <f>C$4</f>
         <v>720000</v>
       </c>
       <c r="D28">
@@ -1273,6 +1294,7 @@
         <v>4</v>
       </c>
       <c r="C29">
+        <f>C$5</f>
         <v>1800000</v>
       </c>
       <c r="D29">
@@ -1290,7 +1312,8 @@
         <v>5</v>
       </c>
       <c r="C30">
-        <v>3600000</v>
+        <f>C$6</f>
+        <v>3700000</v>
       </c>
       <c r="D30">
         <v>0.23</v>
@@ -1307,7 +1330,8 @@
         <v>6</v>
       </c>
       <c r="C31">
-        <v>4800000</v>
+        <f>C$7</f>
+        <v>5800000</v>
       </c>
       <c r="D31">
         <v>0.30499999999999999</v>
@@ -1346,6 +1370,7 @@
         <v>30</v>
       </c>
       <c r="B2">
+        <f>Tabelas_Referencia!C7</f>
         <v>5800000</v>
       </c>
       <c r="C2" t="s">
@@ -1357,7 +1382,8 @@
         <v>32</v>
       </c>
       <c r="B3">
-        <v>3620000</v>
+        <f>Tabelas_Referencia!C6</f>
+        <v>3700000</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>

</xml_diff>